<commit_message>
fix: links Mastodon y datos erróneos
- AppSection: mastodon href construido correctamente desde user@instancia
  → https://instancia/@usuario (antes usaba el handle crudo como URL)
- Eliminado handle inválido de IU (faltaba la instancia; check_activity
  lo ignoraba silenciosamente)
- Eliminado handle erróneo de Marga Prohens Rigo (tenía la cuenta de IU)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dataset/datosfinales.xlsx
+++ b/dataset/datosfinales.xlsx
@@ -27725,16 +27725,6 @@
           <t>2026-05-12</t>
         </is>
       </c>
-      <c r="G692" t="inlineStr">
-        <is>
-          <t>izquierda_unida</t>
-        </is>
-      </c>
-      <c r="H692" t="inlineStr">
-        <is>
-          <t>2026-04-22</t>
-        </is>
-      </c>
       <c r="I692" t="inlineStr">
         <is>
           <t>comunicacion@izquierda-unida.es</t>
@@ -29946,11 +29936,6 @@
       <c r="F751" t="inlineStr">
         <is>
           <t>2024-11-28</t>
-        </is>
-      </c>
-      <c r="G751" t="inlineStr">
-        <is>
-          <t>izquierda_unida</t>
         </is>
       </c>
       <c r="I751" t="inlineStr">

</xml_diff>

<commit_message>
datos: Mastodon IU + diputados Sumar; fix URL construcción Mastodon
- Añadido izquierda_unida@mastodon.social (Izquierda Unida, partidos)
- Añadido enriquesantiago@mastodon.social (Santiago Romero, Enrique Fernando)
  → bio confirma: "Diputado de Izquierda Unida en el Grupo Plurinacional"
- Añadido franciscosierra@mastodon.social (Sierra Caballero, Francisco)
  → catedrático de Comunicación, director FIM, alineado con IU/Sumar
- Actividad verificada: IU activa 2026-05-12, Enrique activo 2026-05-14,
  Francisco activo 2026-04-07
- AppSection: mastodonHref() construye URL correcta desde user@instancia

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dataset/datosfinales.xlsx
+++ b/dataset/datosfinales.xlsx
@@ -15946,6 +15946,16 @@
           <t>2026-05-14</t>
         </is>
       </c>
+      <c r="G365" t="inlineStr">
+        <is>
+          <t>enriquesantiago@mastodon.social</t>
+        </is>
+      </c>
+      <c r="H365" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
       <c r="I365" t="inlineStr">
         <is>
           <t>enrique.santiago@congreso.es</t>
@@ -16344,6 +16354,16 @@
           <t>2026-04-17</t>
         </is>
       </c>
+      <c r="G374" t="inlineStr">
+        <is>
+          <t>franciscosierra@mastodon.social</t>
+        </is>
+      </c>
+      <c r="H374" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
       <c r="I374" t="inlineStr">
         <is>
           <t>francisco.sierra@congreso.es</t>
@@ -27721,6 +27741,16 @@
         </is>
       </c>
       <c r="F692" t="inlineStr">
+        <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="G692" t="inlineStr">
+        <is>
+          <t>izquierda_unida@mastodon.social</t>
+        </is>
+      </c>
+      <c r="H692" t="inlineStr">
         <is>
           <t>2026-05-12</t>
         </is>

</xml_diff>

<commit_message>
datos: Bluesky Teslem Andala; tooltip por delegación de eventos (position:fixed)
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dataset/datosfinales.xlsx
+++ b/dataset/datosfinales.xlsx
@@ -3860,6 +3860,16 @@
           <t>Thu May 14</t>
         </is>
       </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>teshsidi.bsky.social</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>2026-04-23</t>
+        </is>
+      </c>
       <c r="I87" t="inlineStr">
         <is>
           <t>teshsidi@congreso.es</t>

</xml_diff>

<commit_message>
fix: Bluesky Carla Antonelli (senadora); tooltip JS puro sin TypeScript
- carladelgado.bsky.social era periodista UK → corregida a carlaantonelli.bsky.social
- Tooltip reescrito en JS vanilla, sin casts TypeScript que podían fallar silenciosamente

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dataset/datosfinales.xlsx
+++ b/dataset/datosfinales.xlsx
@@ -20630,12 +20630,12 @@
       </c>
       <c r="E486" t="inlineStr">
         <is>
-          <t>carladelgado.bsky.social</t>
+          <t>carlaantonelli.bsky.social</t>
         </is>
       </c>
       <c r="F486" t="inlineStr">
         <is>
-          <t>2025-03-30</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="K486" t="inlineStr">

</xml_diff>

<commit_message>
fix: 5 handles Bluesky erróneos; tooltip sobrevive navegación con view transitions
Datos:
- lyadelestado + seacabolafiesta: faltaba .bsky.social
- santirodriguez.bsky.social: era piloto/modelo, no el diputado → eliminado
- joseframirez.bsky.social, jorgemtnez.bsky.social: handles inválidos (400) → eliminados

Tooltip:
- window._barTipListeners evita duplicar listeners entre navegaciones
- getTip() recrea el div si view transitions lo elimina del body
- astro:page-load garantiza que el div esté disponible tras cada transición

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dataset/datosfinales.xlsx
+++ b/dataset/datosfinales.xlsx
@@ -1946,7 +1946,7 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>lyadelestado</t>
+          <t>lyadelestado.bsky.social</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -14171,16 +14171,6 @@
           <t>Thu May 14</t>
         </is>
       </c>
-      <c r="E325" t="inlineStr">
-        <is>
-          <t>joseframirez.bsky.social</t>
-        </is>
-      </c>
-      <c r="F325" t="inlineStr">
-        <is>
-          <t>404</t>
-        </is>
-      </c>
       <c r="I325" t="inlineStr">
         <is>
           <t>jose.ramirez@congreso.es</t>
@@ -14935,16 +14925,6 @@
           <t>Thu May 14</t>
         </is>
       </c>
-      <c r="E342" t="inlineStr">
-        <is>
-          <t>santirodriguez.bsky.social</t>
-        </is>
-      </c>
-      <c r="F342" t="inlineStr">
-        <is>
-          <t>2026-04-20</t>
-        </is>
-      </c>
       <c r="I342" t="inlineStr">
         <is>
           <t>santi.rodriguez@congreso.es</t>
@@ -23559,16 +23539,6 @@
           <t>Martínez Antolín, Jorge Domingo</t>
         </is>
       </c>
-      <c r="E569" t="inlineStr">
-        <is>
-          <t>jorgemtnez.bsky.social</t>
-        </is>
-      </c>
-      <c r="F569" t="inlineStr">
-        <is>
-          <t>404</t>
-        </is>
-      </c>
       <c r="I569" t="inlineStr">
         <is>
           <t>jdomingo.martinez@senado.es</t>
@@ -28296,7 +28266,7 @@
       </c>
       <c r="E709" t="inlineStr">
         <is>
-          <t>seacabolafiesta</t>
+          <t>seacabolafiesta.bsky.social</t>
         </is>
       </c>
       <c r="F709" t="inlineStr">

</xml_diff>

<commit_message>
fix: Bluesky Rufián gabrielrufian → grufian; confirmar cuentas sin bio por posts
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dataset/datosfinales.xlsx
+++ b/dataset/datosfinales.xlsx
@@ -15421,7 +15421,12 @@
       </c>
       <c r="E354" t="inlineStr">
         <is>
-          <t>gabrielrufian.bsky.social</t>
+          <t>grufian.bsky.social</t>
+        </is>
+      </c>
+      <c r="F354" t="inlineStr">
+        <is>
+          <t>2025-11-04</t>
         </is>
       </c>
       <c r="I354" t="inlineStr">

</xml_diff>

<commit_message>
datos: actualización mensual 2026-08-01
</commit_message>
<xml_diff>
--- a/dataset/datosfinales.xlsx
+++ b/dataset/datosfinales.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -584,7 +584,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -626,7 +626,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -668,7 +668,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -747,7 +747,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -821,7 +821,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -863,7 +863,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -1011,7 +1011,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1090,7 +1090,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1174,7 +1174,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1216,7 +1216,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -1332,7 +1332,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -1416,7 +1416,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -1495,7 +1495,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -1542,7 +1542,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -1589,7 +1589,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
@@ -1710,7 +1710,7 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
@@ -1831,7 +1831,7 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
@@ -1878,7 +1878,7 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
@@ -1962,7 +1962,7 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
@@ -2172,7 +2172,7 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
@@ -2256,7 +2256,7 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
@@ -2369,7 +2369,7 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
@@ -2783,7 +2783,7 @@
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="J70" t="inlineStr">
@@ -2827,7 +2827,7 @@
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="J72" t="inlineStr">
@@ -3040,7 +3040,7 @@
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="J81" t="inlineStr">
@@ -3114,7 +3114,7 @@
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="J83" t="inlineStr">
@@ -3454,7 +3454,7 @@
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="J93" t="inlineStr">
@@ -3528,7 +3528,7 @@
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="J95" t="inlineStr">
@@ -3718,7 +3718,7 @@
       </c>
       <c r="F100" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="J100" t="inlineStr">
@@ -3836,7 +3836,7 @@
       </c>
       <c r="F104" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="J104" t="inlineStr">
@@ -4008,7 +4008,7 @@
       </c>
       <c r="F110" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="J110" t="inlineStr">
@@ -4050,7 +4050,7 @@
       </c>
       <c r="F111" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="J111" t="inlineStr">
@@ -4092,7 +4092,7 @@
       </c>
       <c r="F112" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="J112" t="inlineStr">
@@ -4262,7 +4262,7 @@
       </c>
       <c r="F117" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="J117" t="inlineStr">
@@ -4304,7 +4304,7 @@
       </c>
       <c r="F118" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="J118" t="inlineStr">
@@ -4346,7 +4346,7 @@
       </c>
       <c r="F119" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="J119" t="inlineStr">
@@ -4388,7 +4388,7 @@
       </c>
       <c r="F120" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="J120" t="inlineStr">
@@ -4430,7 +4430,7 @@
       </c>
       <c r="F121" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="J121" t="inlineStr">
@@ -4504,7 +4504,7 @@
       </c>
       <c r="F123" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="J123" t="inlineStr">
@@ -4578,7 +4578,7 @@
       </c>
       <c r="F125" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="J125" t="inlineStr">
@@ -4620,7 +4620,7 @@
       </c>
       <c r="F126" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="J126" t="inlineStr">
@@ -4694,7 +4694,7 @@
       </c>
       <c r="F128" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="J128" t="inlineStr">
@@ -4832,7 +4832,7 @@
       </c>
       <c r="F132" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="J132" t="inlineStr">
@@ -5012,7 +5012,7 @@
       </c>
       <c r="F137" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-26</t>
         </is>
       </c>
       <c r="J137" t="inlineStr">
@@ -5086,7 +5086,7 @@
       </c>
       <c r="F139" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="J139" t="inlineStr">
@@ -5458,7 +5458,7 @@
       </c>
       <c r="F150" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="J150" t="inlineStr">
@@ -6656,7 +6656,7 @@
       </c>
       <c r="F189" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="J189" t="inlineStr">
@@ -7012,7 +7012,7 @@
       </c>
       <c r="F202" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="J202" t="inlineStr">
@@ -7086,7 +7086,7 @@
       </c>
       <c r="F204" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="J204" t="inlineStr">
@@ -7128,7 +7128,7 @@
       </c>
       <c r="F205" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="J205" t="inlineStr">
@@ -7202,7 +7202,7 @@
       </c>
       <c r="F207" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="J207" t="inlineStr">
@@ -7911,6 +7911,11 @@
           <t>centromemorialvt.bsky.social</t>
         </is>
       </c>
+      <c r="F230" t="inlineStr">
+        <is>
+          <t>2025-12-16</t>
+        </is>
+      </c>
       <c r="J230" t="inlineStr">
         <is>
           <t>Fundación Estatal</t>
@@ -8796,7 +8801,7 @@
       </c>
       <c r="F259" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="J259" t="inlineStr">
@@ -9128,7 +9133,7 @@
       </c>
       <c r="F270" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="J270" t="inlineStr">
@@ -9214,7 +9219,7 @@
       </c>
       <c r="F273" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="J273" t="inlineStr">
@@ -9246,7 +9251,7 @@
       </c>
       <c r="F274" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="J274" t="inlineStr">
@@ -9386,7 +9391,7 @@
       </c>
       <c r="F279" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="J279" t="inlineStr">
@@ -9546,7 +9551,7 @@
       </c>
       <c r="F284" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="J284" t="inlineStr">
@@ -9804,7 +9809,7 @@
       </c>
       <c r="F293" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="J293" t="inlineStr">
@@ -9954,7 +9959,7 @@
       </c>
       <c r="F298" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="I298" t="inlineStr">
@@ -9986,7 +9991,7 @@
       </c>
       <c r="F299" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="I299" t="inlineStr">
@@ -10028,7 +10033,7 @@
       </c>
       <c r="F300" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="I300" t="inlineStr">
@@ -10070,7 +10075,7 @@
       </c>
       <c r="F301" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="I301" t="inlineStr">
@@ -10198,7 +10203,7 @@
       </c>
       <c r="F305" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="I305" t="inlineStr">
@@ -10388,7 +10393,7 @@
       </c>
       <c r="F310" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="I310" t="inlineStr">
@@ -10430,7 +10435,7 @@
       </c>
       <c r="F311" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="I311" t="inlineStr">
@@ -10472,7 +10477,7 @@
       </c>
       <c r="F312" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="I312" t="inlineStr">
@@ -10514,7 +10519,7 @@
       </c>
       <c r="F313" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="I313" t="inlineStr">
@@ -10620,7 +10625,7 @@
       </c>
       <c r="F316" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="I316" t="inlineStr">
@@ -10694,7 +10699,7 @@
       </c>
       <c r="F318" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="I318" t="inlineStr">
@@ -10763,7 +10768,7 @@
       </c>
       <c r="F320" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="K320" t="inlineStr">
@@ -11173,7 +11178,7 @@
       </c>
       <c r="F330" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="I330" t="inlineStr">
@@ -11450,7 +11455,7 @@
       </c>
       <c r="F336" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="I336" t="inlineStr">
@@ -11942,7 +11947,7 @@
       </c>
       <c r="F347" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="K347" t="inlineStr">
@@ -12335,7 +12340,7 @@
       </c>
       <c r="F356" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="I356" t="inlineStr">
@@ -12681,7 +12686,7 @@
       </c>
       <c r="F364" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="K364" t="inlineStr">
@@ -13689,7 +13694,7 @@
       </c>
       <c r="F388" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="I388" t="inlineStr">
@@ -14685,7 +14690,7 @@
       </c>
       <c r="F411" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="I411" t="inlineStr">
@@ -15787,7 +15792,7 @@
       </c>
       <c r="F437" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="I437" t="inlineStr">
@@ -15955,7 +15960,7 @@
       </c>
       <c r="F441" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="I441" t="inlineStr">
@@ -16091,7 +16096,7 @@
       </c>
       <c r="F444" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="I444" t="inlineStr">
@@ -16803,7 +16808,7 @@
       </c>
       <c r="F460" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="I460" t="inlineStr">
@@ -17092,7 +17097,7 @@
       </c>
       <c r="F467" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="I467" t="inlineStr">
@@ -17836,7 +17841,7 @@
       </c>
       <c r="F484" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="I484" t="inlineStr">
@@ -18308,7 +18313,7 @@
       </c>
       <c r="F495" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="I495" t="inlineStr">
@@ -18402,7 +18407,7 @@
       </c>
       <c r="F497" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="I497" t="inlineStr">
@@ -18449,7 +18454,7 @@
       </c>
       <c r="F498" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="I498" t="inlineStr">
@@ -18815,7 +18820,7 @@
       </c>
       <c r="F506" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="I506" t="inlineStr">
@@ -20312,7 +20317,7 @@
       </c>
       <c r="F542" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="I542" t="inlineStr">
@@ -23453,7 +23458,7 @@
       </c>
       <c r="F615" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="I615" t="inlineStr">
@@ -23547,7 +23552,7 @@
       </c>
       <c r="F617" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="G617" t="inlineStr">
@@ -23557,7 +23562,7 @@
       </c>
       <c r="H617" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="I617" t="inlineStr">
@@ -23955,7 +23960,7 @@
       </c>
       <c r="F626" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="G626" t="inlineStr">
@@ -24153,7 +24158,7 @@
       </c>
       <c r="F630" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="I630" t="inlineStr">
@@ -24605,7 +24610,7 @@
       </c>
       <c r="F641" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="I641" t="inlineStr">
@@ -25544,7 +25549,7 @@
       </c>
       <c r="F663" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="I663" t="inlineStr">
@@ -28219,7 +28224,7 @@
       </c>
       <c r="F738" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="K738" t="inlineStr">
@@ -28451,7 +28456,7 @@
       </c>
       <c r="F744" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="I744" t="inlineStr">
@@ -28582,7 +28587,7 @@
       </c>
       <c r="F747" t="inlineStr">
         <is>
-          <t>2026-03-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="K747" t="inlineStr">
@@ -31703,7 +31708,7 @@
       </c>
       <c r="F840" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="I840" t="inlineStr">
@@ -34906,7 +34911,7 @@
       </c>
       <c r="F934" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="I934" t="inlineStr">
@@ -34970,7 +34975,7 @@
       </c>
       <c r="F936" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="I936" t="inlineStr">
@@ -35007,7 +35012,7 @@
       </c>
       <c r="F937" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="I937" t="inlineStr">
@@ -35081,7 +35086,7 @@
       </c>
       <c r="F939" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="I939" t="inlineStr">
@@ -35209,7 +35214,7 @@
       </c>
       <c r="F943" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="I943" t="inlineStr">
@@ -35246,7 +35251,7 @@
       </c>
       <c r="F944" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="G944" t="inlineStr">
@@ -35256,7 +35261,7 @@
       </c>
       <c r="H944" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="I944" t="inlineStr">
@@ -35367,7 +35372,7 @@
       </c>
       <c r="F947" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="I947" t="inlineStr">
@@ -35404,7 +35409,7 @@
       </c>
       <c r="F948" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="I948" t="inlineStr">
@@ -36449,7 +36454,7 @@
       </c>
       <c r="F978" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="I978" t="inlineStr">
@@ -37747,7 +37752,7 @@
       </c>
       <c r="F1012" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="I1012" t="inlineStr">
@@ -40191,7 +40196,7 @@
       </c>
       <c r="F1084" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="K1084" t="inlineStr">
@@ -41307,7 +41312,7 @@
       </c>
       <c r="F1117" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="K1117" t="inlineStr">
@@ -41864,7 +41869,7 @@
       </c>
       <c r="F1133" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="K1133" t="inlineStr">
@@ -43354,7 +43359,7 @@
       </c>
       <c r="F1178" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="K1178" t="inlineStr">
@@ -46447,7 +46452,7 @@
       </c>
       <c r="F1267" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="K1267" t="inlineStr">
@@ -48729,7 +48734,7 @@
       </c>
       <c r="F1333" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="I1333" t="inlineStr">
@@ -48771,7 +48776,7 @@
       </c>
       <c r="F1334" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="I1334" t="inlineStr">
@@ -48813,7 +48818,7 @@
       </c>
       <c r="F1335" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="I1335" t="inlineStr">
@@ -48961,7 +48966,7 @@
       </c>
       <c r="F1339" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="I1339" t="inlineStr">
@@ -49008,7 +49013,7 @@
       </c>
       <c r="F1340" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="I1340" t="inlineStr">
@@ -49082,7 +49087,7 @@
       </c>
       <c r="F1342" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="I1342" t="inlineStr">
@@ -49161,7 +49166,7 @@
       </c>
       <c r="F1344" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="I1344" t="inlineStr">
@@ -49245,7 +49250,7 @@
       </c>
       <c r="F1346" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="I1346" t="inlineStr">
@@ -49324,7 +49329,7 @@
       </c>
       <c r="F1348" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="I1348" t="inlineStr">
@@ -49403,7 +49408,7 @@
       </c>
       <c r="F1350" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="I1350" t="inlineStr">
@@ -49482,7 +49487,7 @@
       </c>
       <c r="F1352" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="I1352" t="inlineStr">
@@ -49556,7 +49561,7 @@
       </c>
       <c r="F1354" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="I1354" t="inlineStr">
@@ -49640,7 +49645,7 @@
       </c>
       <c r="F1356" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="I1356" t="inlineStr">
@@ -49751,7 +49756,7 @@
       </c>
       <c r="F1359" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="I1359" t="inlineStr">
@@ -49825,7 +49830,7 @@
       </c>
       <c r="F1361" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="I1361" t="inlineStr">
@@ -49867,7 +49872,7 @@
       </c>
       <c r="F1362" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="I1362" t="inlineStr">
@@ -49909,7 +49914,7 @@
       </c>
       <c r="F1363" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="I1363" t="inlineStr">
@@ -49951,7 +49956,7 @@
       </c>
       <c r="F1364" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="I1364" t="inlineStr">
@@ -49993,7 +49998,7 @@
       </c>
       <c r="F1365" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="I1365" t="inlineStr">
@@ -50035,7 +50040,7 @@
       </c>
       <c r="F1366" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="I1366" t="inlineStr">
@@ -50077,7 +50082,7 @@
       </c>
       <c r="F1367" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="I1367" t="inlineStr">
@@ -50119,7 +50124,7 @@
       </c>
       <c r="F1368" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="I1368" t="inlineStr">
@@ -50161,7 +50166,7 @@
       </c>
       <c r="F1369" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="I1369" t="inlineStr">
@@ -50203,7 +50208,7 @@
       </c>
       <c r="F1370" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="I1370" t="inlineStr">
@@ -50245,7 +50250,7 @@
       </c>
       <c r="F1371" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="I1371" t="inlineStr">
@@ -50287,7 +50292,7 @@
       </c>
       <c r="F1372" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="I1372" t="inlineStr">
@@ -50329,7 +50334,7 @@
       </c>
       <c r="F1373" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="I1373" t="inlineStr">
@@ -50455,7 +50460,7 @@
       </c>
       <c r="F1376" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="I1376" t="inlineStr">
@@ -50497,7 +50502,7 @@
       </c>
       <c r="F1377" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="I1377" t="inlineStr">
@@ -50539,7 +50544,7 @@
       </c>
       <c r="F1378" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="I1378" t="inlineStr">
@@ -50581,7 +50586,7 @@
       </c>
       <c r="F1379" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="I1379" t="inlineStr">
@@ -50623,7 +50628,7 @@
       </c>
       <c r="F1380" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="I1380" t="inlineStr">
@@ -50665,7 +50670,7 @@
       </c>
       <c r="F1381" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="I1381" t="inlineStr">
@@ -50707,7 +50712,7 @@
       </c>
       <c r="F1382" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="I1382" t="inlineStr">
@@ -50982,7 +50987,7 @@
       </c>
       <c r="F1392" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="J1392" t="inlineStr">
@@ -51019,7 +51024,7 @@
       </c>
       <c r="F1393" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="J1393" t="inlineStr">

</xml_diff>

<commit_message>
fix: no sobrescribe la fecha real de última actividad en Twitter/X con 404
Antes se perdía para siempre la fecha del último post cuando una cuenta
desaparecía. Ahora el 404 se registra en una columna de estado aparte y
se añade también una columna de fecha de última consulta.
</commit_message>
<xml_diff>
--- a/dataset/datosfinales.xlsx
+++ b/dataset/datosfinales.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P1396"/>
+  <dimension ref="A1:R1396"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -518,6 +518,16 @@
           <t>Invente</t>
         </is>
       </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>Twitter Última consulta</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>Twitter Estado</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -3309,24 +3319,24 @@
           <t>DeleGobCataluna</t>
         </is>
       </c>
-      <c r="D89" t="inlineStr">
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>delegobcataluna.bsky.social</t>
+        </is>
+      </c>
+      <c r="J89" t="inlineStr">
+        <is>
+          <t>Delegación del Gobierno</t>
+        </is>
+      </c>
+      <c r="N89" t="inlineStr">
+        <is>
+          <t>Cataluña</t>
+        </is>
+      </c>
+      <c r="R89" t="inlineStr">
         <is>
           <t>404</t>
-        </is>
-      </c>
-      <c r="E89" t="inlineStr">
-        <is>
-          <t>delegobcataluna.bsky.social</t>
-        </is>
-      </c>
-      <c r="J89" t="inlineStr">
-        <is>
-          <t>Delegación del Gobierno</t>
-        </is>
-      </c>
-      <c r="N89" t="inlineStr">
-        <is>
-          <t>Cataluña</t>
         </is>
       </c>
     </row>
@@ -5382,19 +5392,19 @@
           <t>Isdefe_</t>
         </is>
       </c>
-      <c r="D148" t="inlineStr">
+      <c r="J148" t="inlineStr">
+        <is>
+          <t>Sociedad Mercantil Estatal</t>
+        </is>
+      </c>
+      <c r="P148" t="inlineStr">
+        <is>
+          <t>INV00003446</t>
+        </is>
+      </c>
+      <c r="R148" t="inlineStr">
         <is>
           <t>404</t>
-        </is>
-      </c>
-      <c r="J148" t="inlineStr">
-        <is>
-          <t>Sociedad Mercantil Estatal</t>
-        </is>
-      </c>
-      <c r="P148" t="inlineStr">
-        <is>
-          <t>INV00003446</t>
         </is>
       </c>
     </row>
@@ -7574,19 +7584,19 @@
           <t>SevillaZF</t>
         </is>
       </c>
-      <c r="D219" t="inlineStr">
+      <c r="J219" t="inlineStr">
+        <is>
+          <t>Entidad de Derecho Público</t>
+        </is>
+      </c>
+      <c r="P219" t="inlineStr">
+        <is>
+          <t>INV00001469</t>
+        </is>
+      </c>
+      <c r="R219" t="inlineStr">
         <is>
           <t>404</t>
-        </is>
-      </c>
-      <c r="J219" t="inlineStr">
-        <is>
-          <t>Entidad de Derecho Público</t>
-        </is>
-      </c>
-      <c r="P219" t="inlineStr">
-        <is>
-          <t>INV00001469</t>
         </is>
       </c>
     </row>
@@ -7739,19 +7749,19 @@
           <t>ENSAonline</t>
         </is>
       </c>
-      <c r="D224" t="inlineStr">
+      <c r="J224" t="inlineStr">
+        <is>
+          <t>Sociedad Mercantil Estatal</t>
+        </is>
+      </c>
+      <c r="P224" t="inlineStr">
+        <is>
+          <t>INV00002097</t>
+        </is>
+      </c>
+      <c r="R224" t="inlineStr">
         <is>
           <t>404</t>
-        </is>
-      </c>
-      <c r="J224" t="inlineStr">
-        <is>
-          <t>Sociedad Mercantil Estatal</t>
-        </is>
-      </c>
-      <c r="P224" t="inlineStr">
-        <is>
-          <t>INV00002097</t>
         </is>
       </c>
     </row>
@@ -8917,19 +8927,19 @@
           <t>INSS_oficial</t>
         </is>
       </c>
-      <c r="D263" t="inlineStr">
+      <c r="J263" t="inlineStr">
+        <is>
+          <t>Entidad Gestora de la S.S.</t>
+        </is>
+      </c>
+      <c r="P263" t="inlineStr">
+        <is>
+          <t>INV00003732</t>
+        </is>
+      </c>
+      <c r="R263" t="inlineStr">
         <is>
           <t>404</t>
-        </is>
-      </c>
-      <c r="J263" t="inlineStr">
-        <is>
-          <t>Entidad Gestora de la S.S.</t>
-        </is>
-      </c>
-      <c r="P263" t="inlineStr">
-        <is>
-          <t>INV00003732</t>
         </is>
       </c>
     </row>
@@ -11003,29 +11013,29 @@
           <t>jagirretxea</t>
         </is>
       </c>
-      <c r="D326" t="inlineStr">
+      <c r="I326" t="inlineStr">
+        <is>
+          <t>agirretxea@congreso.es</t>
+        </is>
+      </c>
+      <c r="K326" t="inlineStr">
+        <is>
+          <t>Diputado/a</t>
+        </is>
+      </c>
+      <c r="L326" t="inlineStr">
+        <is>
+          <t>Grupo Parlamentario Vasco (EAJ-PNV)</t>
+        </is>
+      </c>
+      <c r="M326" t="inlineStr">
+        <is>
+          <t>Gipuzkoa</t>
+        </is>
+      </c>
+      <c r="R326" t="inlineStr">
         <is>
           <t>404</t>
-        </is>
-      </c>
-      <c r="I326" t="inlineStr">
-        <is>
-          <t>agirretxea@congreso.es</t>
-        </is>
-      </c>
-      <c r="K326" t="inlineStr">
-        <is>
-          <t>Diputado/a</t>
-        </is>
-      </c>
-      <c r="L326" t="inlineStr">
-        <is>
-          <t>Grupo Parlamentario Vasco (EAJ-PNV)</t>
-        </is>
-      </c>
-      <c r="M326" t="inlineStr">
-        <is>
-          <t>Gipuzkoa</t>
         </is>
       </c>
     </row>
@@ -11443,39 +11453,39 @@
           <t>AlonsoCantorne</t>
         </is>
       </c>
-      <c r="D336" t="inlineStr">
+      <c r="E336" t="inlineStr">
+        <is>
+          <t>alonsocantorne.bsky.social</t>
+        </is>
+      </c>
+      <c r="F336" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="I336" t="inlineStr">
+        <is>
+          <t>alonso.cantorne@congreso.es</t>
+        </is>
+      </c>
+      <c r="K336" t="inlineStr">
+        <is>
+          <t>Diputado/a</t>
+        </is>
+      </c>
+      <c r="L336" t="inlineStr">
+        <is>
+          <t>Grupo Parlamentario Plurinacional SUMAR</t>
+        </is>
+      </c>
+      <c r="M336" t="inlineStr">
+        <is>
+          <t>Tarragona</t>
+        </is>
+      </c>
+      <c r="R336" t="inlineStr">
         <is>
           <t>404</t>
-        </is>
-      </c>
-      <c r="E336" t="inlineStr">
-        <is>
-          <t>alonsocantorne.bsky.social</t>
-        </is>
-      </c>
-      <c r="F336" t="inlineStr">
-        <is>
-          <t>2026-08-03</t>
-        </is>
-      </c>
-      <c r="I336" t="inlineStr">
-        <is>
-          <t>alonso.cantorne@congreso.es</t>
-        </is>
-      </c>
-      <c r="K336" t="inlineStr">
-        <is>
-          <t>Diputado/a</t>
-        </is>
-      </c>
-      <c r="L336" t="inlineStr">
-        <is>
-          <t>Grupo Parlamentario Plurinacional SUMAR</t>
-        </is>
-      </c>
-      <c r="M336" t="inlineStr">
-        <is>
-          <t>Tarragona</t>
         </is>
       </c>
     </row>
@@ -21565,29 +21575,29 @@
           <t>OscarRamajoPra</t>
         </is>
       </c>
-      <c r="D572" t="inlineStr">
+      <c r="I572" t="inlineStr">
+        <is>
+          <t>oscar.ramajo@congreso.es</t>
+        </is>
+      </c>
+      <c r="K572" t="inlineStr">
+        <is>
+          <t>Diputado/a</t>
+        </is>
+      </c>
+      <c r="L572" t="inlineStr">
+        <is>
+          <t>Grupo Parlamentario Popular en el Congreso</t>
+        </is>
+      </c>
+      <c r="M572" t="inlineStr">
+        <is>
+          <t>Zamora</t>
+        </is>
+      </c>
+      <c r="R572" t="inlineStr">
         <is>
           <t>404</t>
-        </is>
-      </c>
-      <c r="I572" t="inlineStr">
-        <is>
-          <t>oscar.ramajo@congreso.es</t>
-        </is>
-      </c>
-      <c r="K572" t="inlineStr">
-        <is>
-          <t>Diputado/a</t>
-        </is>
-      </c>
-      <c r="L572" t="inlineStr">
-        <is>
-          <t>Grupo Parlamentario Popular en el Congreso</t>
-        </is>
-      </c>
-      <c r="M572" t="inlineStr">
-        <is>
-          <t>Zamora</t>
         </is>
       </c>
     </row>
@@ -24353,27 +24363,32 @@
       </c>
       <c r="D635" t="inlineStr">
         <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="I635" t="inlineStr">
+        <is>
+          <t>carlos.sanchezojeda@congreso.es</t>
+        </is>
+      </c>
+      <c r="K635" t="inlineStr">
+        <is>
+          <t>Diputado/a</t>
+        </is>
+      </c>
+      <c r="L635" t="inlineStr">
+        <is>
+          <t>Grupo Parlamentario Popular en el Congreso</t>
+        </is>
+      </c>
+      <c r="M635" t="inlineStr">
+        <is>
+          <t>Palmas (Las)</t>
+        </is>
+      </c>
+      <c r="R635" t="inlineStr">
+        <is>
           <t>404</t>
-        </is>
-      </c>
-      <c r="I635" t="inlineStr">
-        <is>
-          <t>carlos.sanchezojeda@congreso.es</t>
-        </is>
-      </c>
-      <c r="K635" t="inlineStr">
-        <is>
-          <t>Diputado/a</t>
-        </is>
-      </c>
-      <c r="L635" t="inlineStr">
-        <is>
-          <t>Grupo Parlamentario Popular en el Congreso</t>
-        </is>
-      </c>
-      <c r="M635" t="inlineStr">
-        <is>
-          <t>Palmas (Las)</t>
         </is>
       </c>
     </row>
@@ -28895,24 +28910,24 @@
           <t>marilo_flores91</t>
         </is>
       </c>
-      <c r="D757" t="inlineStr">
+      <c r="I757" t="inlineStr">
+        <is>
+          <t>mdolores.flores@senado.es</t>
+        </is>
+      </c>
+      <c r="K757" t="inlineStr">
+        <is>
+          <t>Senador/a</t>
+        </is>
+      </c>
+      <c r="L757" t="inlineStr">
+        <is>
+          <t>GPS</t>
+        </is>
+      </c>
+      <c r="R757" t="inlineStr">
         <is>
           <t>404</t>
-        </is>
-      </c>
-      <c r="I757" t="inlineStr">
-        <is>
-          <t>mdolores.flores@senado.es</t>
-        </is>
-      </c>
-      <c r="K757" t="inlineStr">
-        <is>
-          <t>Senador/a</t>
-        </is>
-      </c>
-      <c r="L757" t="inlineStr">
-        <is>
-          <t>GPS</t>
         </is>
       </c>
     </row>
@@ -32953,24 +32968,24 @@
           <t>PRojoNoguera</t>
         </is>
       </c>
-      <c r="D876" t="inlineStr">
+      <c r="I876" t="inlineStr">
+        <is>
+          <t>pilar.rojo@senado.es</t>
+        </is>
+      </c>
+      <c r="K876" t="inlineStr">
+        <is>
+          <t>Senador/a</t>
+        </is>
+      </c>
+      <c r="L876" t="inlineStr">
+        <is>
+          <t>GPP</t>
+        </is>
+      </c>
+      <c r="R876" t="inlineStr">
         <is>
           <t>404</t>
-        </is>
-      </c>
-      <c r="I876" t="inlineStr">
-        <is>
-          <t>pilar.rojo@senado.es</t>
-        </is>
-      </c>
-      <c r="K876" t="inlineStr">
-        <is>
-          <t>Senador/a</t>
-        </is>
-      </c>
-      <c r="L876" t="inlineStr">
-        <is>
-          <t>GPP</t>
         </is>
       </c>
     </row>
@@ -38086,24 +38101,24 @@
           <t>ArkauteAkademia</t>
         </is>
       </c>
-      <c r="D1020" t="inlineStr">
+      <c r="K1020" t="inlineStr">
+        <is>
+          <t>Organismo Autónomo</t>
+        </is>
+      </c>
+      <c r="N1020" t="inlineStr">
+        <is>
+          <t>País Vasco</t>
+        </is>
+      </c>
+      <c r="P1020" t="inlineStr">
+        <is>
+          <t>INV00000015</t>
+        </is>
+      </c>
+      <c r="R1020" t="inlineStr">
         <is>
           <t>404</t>
-        </is>
-      </c>
-      <c r="K1020" t="inlineStr">
-        <is>
-          <t>Organismo Autónomo</t>
-        </is>
-      </c>
-      <c r="N1020" t="inlineStr">
-        <is>
-          <t>País Vasco</t>
-        </is>
-      </c>
-      <c r="P1020" t="inlineStr">
-        <is>
-          <t>INV00000015</t>
         </is>
       </c>
     </row>
@@ -38234,24 +38249,24 @@
           <t>aaconocimiento</t>
         </is>
       </c>
-      <c r="D1024" t="inlineStr">
+      <c r="K1024" t="inlineStr">
+        <is>
+          <t>Agencia</t>
+        </is>
+      </c>
+      <c r="N1024" t="inlineStr">
+        <is>
+          <t>Andalucía</t>
+        </is>
+      </c>
+      <c r="P1024" t="inlineStr">
+        <is>
+          <t>INV00000048</t>
+        </is>
+      </c>
+      <c r="R1024" t="inlineStr">
         <is>
           <t>404</t>
-        </is>
-      </c>
-      <c r="K1024" t="inlineStr">
-        <is>
-          <t>Agencia</t>
-        </is>
-      </c>
-      <c r="N1024" t="inlineStr">
-        <is>
-          <t>Andalucía</t>
-        </is>
-      </c>
-      <c r="P1024" t="inlineStr">
-        <is>
-          <t>INV00000048</t>
         </is>
       </c>
     </row>
@@ -39807,24 +39822,24 @@
           <t>GVAavi</t>
         </is>
       </c>
-      <c r="D1073" t="inlineStr">
+      <c r="K1073" t="inlineStr">
+        <is>
+          <t>Ente Público</t>
+        </is>
+      </c>
+      <c r="N1073" t="inlineStr">
+        <is>
+          <t>Comunitat Valenciana</t>
+        </is>
+      </c>
+      <c r="P1073" t="inlineStr">
+        <is>
+          <t>INV00000153</t>
+        </is>
+      </c>
+      <c r="R1073" t="inlineStr">
         <is>
           <t>404</t>
-        </is>
-      </c>
-      <c r="K1073" t="inlineStr">
-        <is>
-          <t>Ente Público</t>
-        </is>
-      </c>
-      <c r="N1073" t="inlineStr">
-        <is>
-          <t>Comunitat Valenciana</t>
-        </is>
-      </c>
-      <c r="P1073" t="inlineStr">
-        <is>
-          <t>INV00000153</t>
         </is>
       </c>
     </row>
@@ -39982,24 +39997,24 @@
           <t>avpd_dbeb</t>
         </is>
       </c>
-      <c r="D1078" t="inlineStr">
+      <c r="K1078" t="inlineStr">
+        <is>
+          <t>Ente Público</t>
+        </is>
+      </c>
+      <c r="N1078" t="inlineStr">
+        <is>
+          <t>País Vasco</t>
+        </is>
+      </c>
+      <c r="P1078" t="inlineStr">
+        <is>
+          <t>INV00000160</t>
+        </is>
+      </c>
+      <c r="R1078" t="inlineStr">
         <is>
           <t>404</t>
-        </is>
-      </c>
-      <c r="K1078" t="inlineStr">
-        <is>
-          <t>Ente Público</t>
-        </is>
-      </c>
-      <c r="N1078" t="inlineStr">
-        <is>
-          <t>País Vasco</t>
-        </is>
-      </c>
-      <c r="P1078" t="inlineStr">
-        <is>
-          <t>INV00000160</t>
         </is>
       </c>
     </row>
@@ -40019,24 +40034,24 @@
           <t>AugasdeGalicia</t>
         </is>
       </c>
-      <c r="D1079" t="inlineStr">
+      <c r="K1079" t="inlineStr">
+        <is>
+          <t>Entidad Pública Empresarial</t>
+        </is>
+      </c>
+      <c r="N1079" t="inlineStr">
+        <is>
+          <t>Galicia</t>
+        </is>
+      </c>
+      <c r="P1079" t="inlineStr">
+        <is>
+          <t>INV00000186</t>
+        </is>
+      </c>
+      <c r="R1079" t="inlineStr">
         <is>
           <t>404</t>
-        </is>
-      </c>
-      <c r="K1079" t="inlineStr">
-        <is>
-          <t>Entidad Pública Empresarial</t>
-        </is>
-      </c>
-      <c r="N1079" t="inlineStr">
-        <is>
-          <t>Galicia</t>
-        </is>
-      </c>
-      <c r="P1079" t="inlineStr">
-        <is>
-          <t>INV00000186</t>
         </is>
       </c>
     </row>
@@ -41384,24 +41399,24 @@
           <t>CNJCat</t>
         </is>
       </c>
-      <c r="D1119" t="inlineStr">
+      <c r="K1119" t="inlineStr">
+        <is>
+          <t>Ente Público</t>
+        </is>
+      </c>
+      <c r="N1119" t="inlineStr">
+        <is>
+          <t>Catalunya</t>
+        </is>
+      </c>
+      <c r="P1119" t="inlineStr">
+        <is>
+          <t>INV00001313</t>
+        </is>
+      </c>
+      <c r="R1119" t="inlineStr">
         <is>
           <t>404</t>
-        </is>
-      </c>
-      <c r="K1119" t="inlineStr">
-        <is>
-          <t>Ente Público</t>
-        </is>
-      </c>
-      <c r="N1119" t="inlineStr">
-        <is>
-          <t>Catalunya</t>
-        </is>
-      </c>
-      <c r="P1119" t="inlineStr">
-        <is>
-          <t>INV00001313</t>
         </is>
       </c>
     </row>
@@ -41968,24 +41983,24 @@
           <t>EVha_gva</t>
         </is>
       </c>
-      <c r="D1136" t="inlineStr">
+      <c r="K1136" t="inlineStr">
+        <is>
+          <t>Entidad Pública Empresarial</t>
+        </is>
+      </c>
+      <c r="N1136" t="inlineStr">
+        <is>
+          <t>Comunitat Valenciana</t>
+        </is>
+      </c>
+      <c r="P1136" t="inlineStr">
+        <is>
+          <t>INV00002080</t>
+        </is>
+      </c>
+      <c r="R1136" t="inlineStr">
         <is>
           <t>404</t>
-        </is>
-      </c>
-      <c r="K1136" t="inlineStr">
-        <is>
-          <t>Entidad Pública Empresarial</t>
-        </is>
-      </c>
-      <c r="N1136" t="inlineStr">
-        <is>
-          <t>Comunitat Valenciana</t>
-        </is>
-      </c>
-      <c r="P1136" t="inlineStr">
-        <is>
-          <t>INV00002080</t>
         </is>
       </c>
     </row>
@@ -47769,24 +47784,24 @@
           <t>saludextremadur</t>
         </is>
       </c>
-      <c r="D1304" t="inlineStr">
+      <c r="K1304" t="inlineStr">
+        <is>
+          <t>Organismo Autónomo</t>
+        </is>
+      </c>
+      <c r="N1304" t="inlineStr">
+        <is>
+          <t>Extremadura</t>
+        </is>
+      </c>
+      <c r="P1304" t="inlineStr">
+        <is>
+          <t>INV00005050</t>
+        </is>
+      </c>
+      <c r="R1304" t="inlineStr">
         <is>
           <t>404</t>
-        </is>
-      </c>
-      <c r="K1304" t="inlineStr">
-        <is>
-          <t>Organismo Autónomo</t>
-        </is>
-      </c>
-      <c r="N1304" t="inlineStr">
-        <is>
-          <t>Extremadura</t>
-        </is>
-      </c>
-      <c r="P1304" t="inlineStr">
-        <is>
-          <t>INV00005050</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: aplica a Bluesky y Mastodon la misma protección de fecha que a Twitter/X
Ya no se pisa la fecha real de última actividad con 404. Además se añaden
las fechas crudas de actividad a total.json para que los snapshots
históricos mensuales permitan reconstruir cuándo abandonó cada red cada
cuenta, no solo un booleano activo/inactivo.
</commit_message>
<xml_diff>
--- a/dataset/datosfinales.xlsx
+++ b/dataset/datosfinales.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R1396"/>
+  <dimension ref="A1:V1396"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -528,6 +528,26 @@
           <t>Twitter Estado</t>
         </is>
       </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>Bluesky Última consulta</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>Bluesky Estado</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>Mastodon Última consulta</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>Mastodon Estado</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">

</xml_diff>